<commit_message>
Cancun: cambiar orden propiedades 2 y 3, imagen portada
</commit_message>
<xml_diff>
--- a/backend/imagenes/Cancun Quintana Roo/1/FORMATO_CANCÚN.xlsx
+++ b/backend/imagenes/Cancun Quintana Roo/1/FORMATO_CANCÚN.xlsx
@@ -410,11 +410,11 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Avenida Bonampak Mza 27, Lote 01 - 02, Zona Hotelera, Cancún, Q.R.</t>
+          <t>Boulevard Kukulcan Km 1 Zona Turistica Puerto Cancun, 77500 Cancún, Q.R.</t>
         </is>
       </c>
       <c r="C2" s="3" t="n">
-        <v>43000</v>
+        <v>130000</v>
       </c>
       <c r="D2" s="4" t="n">
         <v>4</v>
@@ -426,24 +426,24 @@
         <v>2</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H2" s="1" t="inlineStr">
         <is>
-          <t>Gym, Alberca y Area de niños</t>
+          <t>Alberca, Cancha de tenis, Cancha de Padel y Gym</t>
         </is>
       </c>
       <c r="I2" s="4" t="n">
-        <v>400</v>
+        <v>330</v>
       </c>
       <c r="J2" s="1" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>Si</t>
         </is>
       </c>
       <c r="K2" s="1" t="inlineStr">
         <is>
-          <t>Sí</t>
+          <t>No</t>
         </is>
       </c>
     </row>
@@ -455,11 +455,11 @@
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
-          <t>Boulevard Kukulcan Km 1 Zona Turistica Puerto Cancun, 77500 Cancún, Q.R.</t>
+          <t>Avenida Bonampak Mza 27, Lote 01 - 02, Zona Hotelera, Cancún, Q.R.</t>
         </is>
       </c>
       <c r="C3" s="3" t="n">
-        <v>130000</v>
+        <v>43000</v>
       </c>
       <c r="D3" s="4" t="n">
         <v>4</v>
@@ -471,24 +471,24 @@
         <v>2</v>
       </c>
       <c r="G3" s="4" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H3" s="1" t="inlineStr">
         <is>
-          <t>Alberca, Cancha de tenis, Cancha de Padel y Gym</t>
+          <t>Gym, Alberca y Area de niños</t>
         </is>
       </c>
       <c r="I3" s="4" t="n">
-        <v>330</v>
+        <v>400</v>
       </c>
       <c r="J3" s="1" t="inlineStr">
         <is>
-          <t>Si</t>
+          <t>Sí</t>
         </is>
       </c>
       <c r="K3" s="1" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Sí</t>
         </is>
       </c>
     </row>

</xml_diff>